<commit_message>
Workbook import: guard against hostile files, xlsx only
- The zip is checked before it is read: unpacked size capped at 64 MB
  (counted while unpacking), at most 1,000 entries, and a plausible
  declared shared-string count, so a small file cannot exhaust memory.
- Cells are streamed and a cell beyond the import's rows or columns
  refuses the file before anything is sized to fit it.
- Reading runs off the request threads.
- Only .xlsx is read; .xls, .xlsb, .ods and Numbers files are asked to be
  saved as .xlsx or CSV, which also catches web pages named .xls.
- The first visible sheet is read; times become 19:30 and numbers show
  as a spreadsheet does; blank rows keep row numbers right.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TADvkW5mvUGedKinXeDUGm
</commit_message>
<xml_diff>
--- a/crates/core-engines/tests/fixtures/roster.xlsx
+++ b/crates/core-engines/tests/fixtures/roster.xlsx
@@ -4,10 +4,11 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lookup" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,9 +50,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -418,39 +420,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Artist Name</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Genre</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Booking Fee</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Next show</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Active</t>
+          <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>y</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Artist Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Booking Fee</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Next show</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Set time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>DJ Kemi</t>
         </is>
       </c>
@@ -467,6 +512,9 @@
       </c>
       <c r="E2" t="b">
         <v>1</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>0.8125</v>
       </c>
     </row>
     <row r="3">
@@ -483,7 +531,7 @@
       <c r="C3" t="n">
         <v>1250.5</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>46575.8125</v>
       </c>
       <c r="E3" t="b">

</xml_diff>